<commit_message>
Final backtest confirmed - all periods profitable - 5.9% avg monthly
</commit_message>
<xml_diff>
--- a/data/backtest_pa_v2.xlsx
+++ b/data/backtest_pa_v2.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,14 +479,14 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46150.15625</v>
+        <v>46153.48958333334</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46150.16666666666</v>
+        <v>46153.5</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -495,35 +495,35 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>4719.697</v>
+        <v>4674.327</v>
       </c>
       <c r="F2" t="n">
-        <v>4720.782</v>
+        <v>4673.294</v>
       </c>
       <c r="G2" t="n">
-        <v>4717.527</v>
+        <v>4677.426000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>21.7</v>
+        <v>-20.66</v>
       </c>
       <c r="K2" t="n">
-        <v>31.7</v>
+        <v>979.34</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46150.32291666666</v>
+        <v>46153.91666666666</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46150.33333333334</v>
+        <v>46153.92708333334</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -536,16 +536,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4708.033</v>
+        <v>4738.909</v>
       </c>
       <c r="F3" t="n">
-        <v>4710.934</v>
+        <v>4739.909</v>
       </c>
       <c r="G3" t="n">
-        <v>4702.231000000001</v>
+        <v>4735.909</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -553,22 +553,22 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>-29.01</v>
+        <v>-20</v>
       </c>
       <c r="K3" t="n">
-        <v>2.69</v>
+        <v>959.34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46150.38541666666</v>
+        <v>46154.60416666666</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46150.39583333334</v>
+        <v>46154.61458333334</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -577,76 +577,76 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4717.994</v>
+        <v>4685.938</v>
       </c>
       <c r="F4" t="n">
-        <v>4720.782</v>
+        <v>4684.938</v>
       </c>
       <c r="G4" t="n">
-        <v>4712.417999999999</v>
+        <v>4688.938</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>55.76</v>
+        <v>-20</v>
       </c>
       <c r="K4" t="n">
-        <v>58.45</v>
+        <v>939.34</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46150.40625</v>
+        <v>46155.41666666666</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46150.42708333334</v>
+        <v>46155.42708333334</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>BOUNCE</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>4711.712</v>
+        <v>4702.409</v>
       </c>
       <c r="F5" t="n">
-        <v>4707.934</v>
+        <v>4704.15</v>
       </c>
       <c r="G5" t="n">
-        <v>4719.268000000001</v>
+        <v>4697.186</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>75.56</v>
+        <v>-34.82</v>
       </c>
       <c r="K5" t="n">
-        <v>134.01</v>
+        <v>904.52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46153.48958333334</v>
+        <v>46155.78125</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46153.5</v>
+        <v>46155.79166666666</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -659,39 +659,39 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4674.327</v>
+        <v>4684.757</v>
       </c>
       <c r="F6" t="n">
-        <v>4673.294</v>
+        <v>4683.757</v>
       </c>
       <c r="G6" t="n">
-        <v>4676.393000000001</v>
+        <v>4687.757</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>-10.33</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
-        <v>123.68</v>
+        <v>964.52</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46153.91666666666</v>
+        <v>46157.51041666666</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46153.92708333334</v>
+        <v>46157.52083333334</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>4738.909</v>
+        <v>4555.162</v>
       </c>
       <c r="F7" t="n">
-        <v>4739.909</v>
+        <v>4554.162</v>
       </c>
       <c r="G7" t="n">
-        <v>4736.909</v>
+        <v>4558.162</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -717,22 +717,22 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="K7" t="n">
-        <v>113.68</v>
+        <v>944.52</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46154.60416666666</v>
+        <v>46160.3125</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46154.61458333334</v>
+        <v>46160.32291666666</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -741,35 +741,35 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>4685.938</v>
+        <v>4549.108</v>
       </c>
       <c r="F8" t="n">
-        <v>4684.938</v>
+        <v>4551.477</v>
       </c>
       <c r="G8" t="n">
-        <v>4687.938</v>
+        <v>4542.001000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>-10</v>
+        <v>142.14</v>
       </c>
       <c r="K8" t="n">
-        <v>103.68</v>
+        <v>1086.66</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46155.41666666666</v>
+        <v>46160.36458333334</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>46155.42708333334</v>
+        <v>46160.375</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -782,16 +782,16 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4702.409</v>
+        <v>4550.047</v>
       </c>
       <c r="F9" t="n">
-        <v>4704.15</v>
+        <v>4551.477</v>
       </c>
       <c r="G9" t="n">
-        <v>4698.927</v>
+        <v>4545.756999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -799,18 +799,18 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>34.82</v>
+        <v>85.8</v>
       </c>
       <c r="K9" t="n">
-        <v>138.5</v>
+        <v>1172.46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46155.78125</v>
+        <v>46160.45833333334</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46155.79166666666</v>
+        <v>46160.46875</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -823,35 +823,35 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>4684.757</v>
+        <v>4539.363</v>
       </c>
       <c r="F10" t="n">
-        <v>4683.757</v>
+        <v>4536.941</v>
       </c>
       <c r="G10" t="n">
-        <v>4686.757</v>
+        <v>4546.629000000002</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>20</v>
+        <v>-48.44</v>
       </c>
       <c r="K10" t="n">
-        <v>158.5</v>
+        <v>1124.02</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46155.84375</v>
+        <v>46160.82291666666</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46155.91666666666</v>
+        <v>46160.83333333334</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -860,20 +860,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>BOUNCE</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>4691.132</v>
+        <v>4558.429</v>
       </c>
       <c r="F11" t="n">
-        <v>4692.823</v>
+        <v>4559.429</v>
       </c>
       <c r="G11" t="n">
-        <v>4687.749999999998</v>
+        <v>4555.429</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -881,40 +881,40 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>-16.91</v>
+        <v>-20</v>
       </c>
       <c r="K11" t="n">
-        <v>141.59</v>
+        <v>1104.02</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46156.59375</v>
+        <v>46161.19791666666</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>46156.60416666666</v>
+        <v>46161.20833333334</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>BOUNCE</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>4691.28</v>
+        <v>4542.255</v>
       </c>
       <c r="F12" t="n">
-        <v>4692.28</v>
+        <v>4541.255</v>
       </c>
       <c r="G12" t="n">
-        <v>4689.28</v>
+        <v>4545.255</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -922,18 +922,18 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="K12" t="n">
-        <v>161.59</v>
+        <v>1164.02</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46157.51041666666</v>
+        <v>46161.51041666666</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>46157.52083333334</v>
+        <v>46161.52083333334</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -946,16 +946,16 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>4555.162</v>
+        <v>4543.307</v>
       </c>
       <c r="F13" t="n">
-        <v>4554.162</v>
+        <v>4542.043</v>
       </c>
       <c r="G13" t="n">
-        <v>4557.162</v>
+        <v>4547.099</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -963,59 +963,59 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>-10</v>
+        <v>-25.28</v>
       </c>
       <c r="K13" t="n">
-        <v>151.59</v>
+        <v>1138.74</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46157.77083333334</v>
+        <v>46162.53125</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>46157.78125</v>
+        <v>46162.54166666666</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>BOUNCE</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4557.443</v>
+        <v>4496.024</v>
       </c>
       <c r="F14" t="n">
-        <v>4556.443</v>
+        <v>4498.683</v>
       </c>
       <c r="G14" t="n">
-        <v>4559.443</v>
+        <v>4488.047000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>20</v>
+        <v>-53.18</v>
       </c>
       <c r="K14" t="n">
-        <v>171.59</v>
+        <v>1085.56</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46160.3125</v>
+        <v>46162.77083333334</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>46160.32291666666</v>
+        <v>46162.78125</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1028,39 +1028,39 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>4549.108</v>
+        <v>4537.104</v>
       </c>
       <c r="F15" t="n">
-        <v>4551.477</v>
+        <v>4539.78</v>
       </c>
       <c r="G15" t="n">
-        <v>4544.370000000001</v>
+        <v>4529.076000000002</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>47.38</v>
+        <v>-53.52</v>
       </c>
       <c r="K15" t="n">
-        <v>218.97</v>
+        <v>1032.04</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46160.36458333334</v>
+        <v>46163.4375</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>46160.375</v>
+        <v>46163.44791666666</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1069,35 +1069,35 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>4550.047</v>
+        <v>4516.922</v>
       </c>
       <c r="F16" t="n">
-        <v>4551.477</v>
+        <v>4515.922</v>
       </c>
       <c r="G16" t="n">
-        <v>4547.186999999999</v>
+        <v>4519.922</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>28.6</v>
+        <v>-20</v>
       </c>
       <c r="K16" t="n">
-        <v>247.57</v>
+        <v>1012.04</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46160.45833333334</v>
+        <v>46163.59375</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>46160.46875</v>
+        <v>46163.60416666666</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1110,39 +1110,39 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>4539.363</v>
+        <v>4507.284</v>
       </c>
       <c r="F17" t="n">
-        <v>4536.941</v>
+        <v>4506.284</v>
       </c>
       <c r="G17" t="n">
-        <v>4544.207000000001</v>
+        <v>4510.284</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>-24.22</v>
+        <v>60</v>
       </c>
       <c r="K17" t="n">
-        <v>223.35</v>
+        <v>1072.04</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46160.82291666666</v>
+        <v>46164.01041666666</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>46160.83333333334</v>
+        <v>46164.03125</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1151,16 +1151,16 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>4558.429</v>
+        <v>4536.073</v>
       </c>
       <c r="F18" t="n">
-        <v>4559.429</v>
+        <v>4533.314</v>
       </c>
       <c r="G18" t="n">
-        <v>4556.429</v>
+        <v>4544.35</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1168,18 +1168,18 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>-10</v>
+        <v>-55.18</v>
       </c>
       <c r="K18" t="n">
-        <v>213.35</v>
+        <v>1016.86</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46161.19791666666</v>
+        <v>46164.47916666666</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>46161.20833333334</v>
+        <v>46164.5</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1192,16 +1192,16 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>4542.255</v>
+        <v>4521.543</v>
       </c>
       <c r="F19" t="n">
-        <v>4541.255</v>
+        <v>4519.324</v>
       </c>
       <c r="G19" t="n">
-        <v>4544.255</v>
+        <v>4528.2</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1209,18 +1209,18 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>20</v>
+        <v>133.14</v>
       </c>
       <c r="K19" t="n">
-        <v>233.35</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46161.51041666666</v>
+        <v>46164.78125</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>46161.52083333334</v>
+        <v>46164.79166666666</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1233,39 +1233,39 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4543.307</v>
+        <v>4515.193</v>
       </c>
       <c r="F20" t="n">
-        <v>4542.043</v>
+        <v>4514.193</v>
       </c>
       <c r="G20" t="n">
-        <v>4545.835</v>
+        <v>4518.193</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>25.28</v>
+        <v>-20</v>
       </c>
       <c r="K20" t="n">
-        <v>258.63</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46162.53125</v>
+        <v>46164.84375</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>46162.54166666666</v>
+        <v>46164.85416666666</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1274,16 +1274,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>4496.024</v>
+        <v>4509.975</v>
       </c>
       <c r="F21" t="n">
-        <v>4498.683</v>
+        <v>4508.619</v>
       </c>
       <c r="G21" t="n">
-        <v>4490.706000000001</v>
+        <v>4514.043000000002</v>
       </c>
       <c r="H21" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1291,18 +1291,18 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>-26.59</v>
+        <v>-27.12</v>
       </c>
       <c r="K21" t="n">
-        <v>232.04</v>
+        <v>1102.88</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46162.77083333334</v>
+        <v>46167.70833333334</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>46162.78125</v>
+        <v>46167.71875</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1315,80 +1315,80 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>4537.104</v>
+        <v>4574.134</v>
       </c>
       <c r="F22" t="n">
-        <v>4539.78</v>
+        <v>4575.134</v>
       </c>
       <c r="G22" t="n">
-        <v>4531.752000000001</v>
+        <v>4571.134</v>
       </c>
       <c r="H22" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>-26.76</v>
+        <v>60</v>
       </c>
       <c r="K22" t="n">
-        <v>205.28</v>
+        <v>1162.88</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46162.92708333334</v>
+        <v>46167.92708333334</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>46162.94791666666</v>
+        <v>46167.94791666666</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>BOUNCE</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>4539.141</v>
+        <v>4572.911</v>
       </c>
       <c r="F23" t="n">
-        <v>4536.78</v>
+        <v>4575.128</v>
       </c>
       <c r="G23" t="n">
-        <v>4543.862999999999</v>
+        <v>4566.260000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>47.22</v>
+        <v>-44.34</v>
       </c>
       <c r="K23" t="n">
-        <v>252.5</v>
+        <v>1118.54</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46163.4375</v>
+        <v>46168.44791666666</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>46163.44791666666</v>
+        <v>46168.46875</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1397,35 +1397,35 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>4516.922</v>
+        <v>4534.564</v>
       </c>
       <c r="F24" t="n">
-        <v>4515.922</v>
+        <v>4536.459</v>
       </c>
       <c r="G24" t="n">
-        <v>4518.922</v>
+        <v>4528.879000000002</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>-10</v>
+        <v>113.7</v>
       </c>
       <c r="K24" t="n">
-        <v>242.5</v>
+        <v>1232.24</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46163.59375</v>
+        <v>46168.67708333334</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>46163.60416666666</v>
+        <v>46168.6875</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1438,39 +1438,39 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>4507.284</v>
+        <v>4507.745</v>
       </c>
       <c r="F25" t="n">
-        <v>4506.284</v>
+        <v>4506.214</v>
       </c>
       <c r="G25" t="n">
-        <v>4509.284</v>
+        <v>4512.338</v>
       </c>
       <c r="H25" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>20</v>
+        <v>-30.62</v>
       </c>
       <c r="K25" t="n">
-        <v>262.5</v>
+        <v>1201.62</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46164.01041666666</v>
+        <v>46169.19791666666</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>46164.03125</v>
+        <v>46169.20833333334</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1479,16 +1479,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>4536.073</v>
+        <v>4510.335</v>
       </c>
       <c r="F26" t="n">
-        <v>4533.314</v>
+        <v>4512.215</v>
       </c>
       <c r="G26" t="n">
-        <v>4541.591</v>
+        <v>4504.695</v>
       </c>
       <c r="H26" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1496,40 +1496,40 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>-27.59</v>
+        <v>-37.6</v>
       </c>
       <c r="K26" t="n">
-        <v>234.91</v>
+        <v>1164.02</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46164.10416666666</v>
+        <v>46169.84375</v>
       </c>
       <c r="B27" s="1" t="n">
-        <v>46164.11458333334</v>
+        <v>46169.91666666666</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>BOUNCE</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>4522.717</v>
+        <v>4455.093</v>
       </c>
       <c r="F27" t="n">
-        <v>4519.633</v>
+        <v>4456.992</v>
       </c>
       <c r="G27" t="n">
-        <v>4528.884999999999</v>
+        <v>4449.395999999999</v>
       </c>
       <c r="H27" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1537,22 +1537,22 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>-30.84</v>
+        <v>-37.98</v>
       </c>
       <c r="K27" t="n">
-        <v>204.07</v>
+        <v>1126.04</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46164.47916666666</v>
+        <v>46171.29166666666</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>46164.5</v>
+        <v>46171.30208333334</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1561,16 +1561,16 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>4521.543</v>
+        <v>4516.425</v>
       </c>
       <c r="F28" t="n">
-        <v>4519.324</v>
+        <v>4518.088</v>
       </c>
       <c r="G28" t="n">
-        <v>4525.981</v>
+        <v>4511.436000000002</v>
       </c>
       <c r="H28" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1578,18 +1578,18 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>44.38</v>
+        <v>99.78</v>
       </c>
       <c r="K28" t="n">
-        <v>248.45</v>
+        <v>1225.82</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46164.78125</v>
+        <v>46171.79166666666</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>46164.79166666666</v>
+        <v>46171.80208333334</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1602,16 +1602,16 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>4515.193</v>
+        <v>4558.357</v>
       </c>
       <c r="F29" t="n">
-        <v>4514.193</v>
+        <v>4556.219</v>
       </c>
       <c r="G29" t="n">
-        <v>4517.193</v>
+        <v>4564.771</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1619,18 +1619,18 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>-10</v>
+        <v>-42.76</v>
       </c>
       <c r="K29" t="n">
-        <v>238.45</v>
+        <v>1183.06</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46164.84375</v>
+        <v>46174.22916666666</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>46164.85416666666</v>
+        <v>46174.25</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1643,16 +1643,16 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>4509.975</v>
+        <v>4519.644</v>
       </c>
       <c r="F30" t="n">
-        <v>4508.619</v>
+        <v>4516.854</v>
       </c>
       <c r="G30" t="n">
-        <v>4512.687000000002</v>
+        <v>4528.014</v>
       </c>
       <c r="H30" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1660,22 +1660,22 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>-13.56</v>
+        <v>-55.8</v>
       </c>
       <c r="K30" t="n">
-        <v>224.89</v>
+        <v>1127.26</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46167.70833333334</v>
+        <v>46174.41666666666</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>46167.71875</v>
+        <v>46174.42708333334</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1684,35 +1684,35 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>4574.134</v>
+        <v>4501.323</v>
       </c>
       <c r="F31" t="n">
-        <v>4575.134</v>
+        <v>4498.514</v>
       </c>
       <c r="G31" t="n">
-        <v>4572.134</v>
+        <v>4509.750000000001</v>
       </c>
       <c r="H31" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>20</v>
+        <v>-56.18</v>
       </c>
       <c r="K31" t="n">
-        <v>244.89</v>
+        <v>1071.08</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46167.92708333334</v>
+        <v>46175.125</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>46167.94791666666</v>
+        <v>46175.13541666666</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1725,16 +1725,16 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>4572.911</v>
+        <v>4488.012</v>
       </c>
       <c r="F32" t="n">
-        <v>4575.128</v>
+        <v>4489.012</v>
       </c>
       <c r="G32" t="n">
-        <v>4568.477000000001</v>
+        <v>4485.012</v>
       </c>
       <c r="H32" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1742,18 +1742,18 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>-22.17</v>
+        <v>-20</v>
       </c>
       <c r="K32" t="n">
-        <v>222.72</v>
+        <v>1051.08</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46168.14583333334</v>
+        <v>46175.38541666666</v>
       </c>
       <c r="B33" s="1" t="n">
-        <v>46168.15625</v>
+        <v>46175.40625</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1762,20 +1762,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>BOUNCE</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>4541.547</v>
+        <v>4526.834</v>
       </c>
       <c r="F33" t="n">
-        <v>4542.547</v>
+        <v>4529.791</v>
       </c>
       <c r="G33" t="n">
-        <v>4539.547</v>
+        <v>4517.962999999999</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1783,22 +1783,22 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>-10</v>
+        <v>-59.14</v>
       </c>
       <c r="K33" t="n">
-        <v>212.72</v>
+        <v>991.9400000000001</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46168.44791666666</v>
+        <v>46175.6875</v>
       </c>
       <c r="B34" s="1" t="n">
-        <v>46168.46875</v>
+        <v>46175.70833333334</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1807,35 +1807,35 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>4534.564</v>
+        <v>4489.918</v>
       </c>
       <c r="F34" t="n">
-        <v>4536.459</v>
+        <v>4488.498</v>
       </c>
       <c r="G34" t="n">
-        <v>4530.774000000001</v>
+        <v>4494.178</v>
       </c>
       <c r="H34" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>37.9</v>
+        <v>-28.4</v>
       </c>
       <c r="K34" t="n">
-        <v>250.62</v>
+        <v>963.54</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46168.67708333334</v>
+        <v>46176.09375</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>46168.6875</v>
+        <v>46176.10416666666</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1848,16 +1848,16 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>4507.745</v>
+        <v>4478.584</v>
       </c>
       <c r="F35" t="n">
-        <v>4506.214</v>
+        <v>4477.146</v>
       </c>
       <c r="G35" t="n">
-        <v>4510.807</v>
+        <v>4482.898</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1865,22 +1865,22 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>30.62</v>
+        <v>86.28</v>
       </c>
       <c r="K35" t="n">
-        <v>281.24</v>
+        <v>1049.82</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46169.19791666666</v>
+        <v>46176.11458333334</v>
       </c>
       <c r="B36" s="1" t="n">
-        <v>46169.20833333334</v>
+        <v>46176.125</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1889,39 +1889,39 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>4510.335</v>
+        <v>4482.089</v>
       </c>
       <c r="F36" t="n">
-        <v>4512.215</v>
+        <v>4480.574</v>
       </c>
       <c r="G36" t="n">
-        <v>4506.575</v>
+        <v>4486.634000000001</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>-18.8</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="K36" t="n">
-        <v>262.44</v>
+        <v>1140.72</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46169.84375</v>
+        <v>46176.28125</v>
       </c>
       <c r="B37" s="1" t="n">
-        <v>46169.91666666666</v>
+        <v>46176.29166666666</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1930,57 +1930,57 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>4455.093</v>
+        <v>4462.83</v>
       </c>
       <c r="F37" t="n">
-        <v>4456.992</v>
+        <v>4460.778</v>
       </c>
       <c r="G37" t="n">
-        <v>4451.294999999999</v>
+        <v>4468.985999999999</v>
       </c>
       <c r="H37" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>-18.99</v>
+        <v>123.12</v>
       </c>
       <c r="K37" t="n">
-        <v>243.45</v>
+        <v>1263.84</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46171.16666666666</v>
+        <v>46176.34375</v>
       </c>
       <c r="B38" s="1" t="n">
-        <v>46171.17708333334</v>
+        <v>46176.35416666666</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>BOUNCE</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>4502.198</v>
+        <v>4457.252</v>
       </c>
       <c r="F38" t="n">
-        <v>4503.198</v>
+        <v>4454.977</v>
       </c>
       <c r="G38" t="n">
-        <v>4500.198</v>
+        <v>4464.077000000002</v>
       </c>
       <c r="H38" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1988,22 +1988,22 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>-10</v>
+        <v>-45.5</v>
       </c>
       <c r="K38" t="n">
-        <v>233.45</v>
+        <v>1218.34</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46171.29166666666</v>
+        <v>46176.41666666666</v>
       </c>
       <c r="B39" s="1" t="n">
-        <v>46171.30208333334</v>
+        <v>46176.42708333334</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2012,35 +2012,35 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>4516.425</v>
+        <v>4462.809</v>
       </c>
       <c r="F39" t="n">
-        <v>4518.088</v>
+        <v>4460.778</v>
       </c>
       <c r="G39" t="n">
-        <v>4513.099000000001</v>
+        <v>4468.902</v>
       </c>
       <c r="H39" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>33.26</v>
+        <v>-40.62</v>
       </c>
       <c r="K39" t="n">
-        <v>266.71</v>
+        <v>1177.72</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46171.53125</v>
+        <v>46176.61458333334</v>
       </c>
       <c r="B40" s="1" t="n">
-        <v>46171.54166666666</v>
+        <v>46176.625</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -2049,20 +2049,20 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>BOUNCE</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>4522.843</v>
+        <v>4457.258</v>
       </c>
       <c r="F40" t="n">
-        <v>4519.299</v>
+        <v>4454.977</v>
       </c>
       <c r="G40" t="n">
-        <v>4529.931</v>
+        <v>4464.101</v>
       </c>
       <c r="H40" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2070,18 +2070,18 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>-35.44</v>
+        <v>-45.62</v>
       </c>
       <c r="K40" t="n">
-        <v>231.27</v>
+        <v>1132.1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46171.79166666666</v>
+        <v>46176.92708333334</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>46171.80208333334</v>
+        <v>46176.9375</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -2094,39 +2094,39 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>4558.357</v>
+        <v>4433.806</v>
       </c>
       <c r="F41" t="n">
-        <v>4556.219</v>
+        <v>4432.129</v>
       </c>
       <c r="G41" t="n">
-        <v>4562.633</v>
+        <v>4438.836999999999</v>
       </c>
       <c r="H41" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>-21.38</v>
+        <v>100.62</v>
       </c>
       <c r="K41" t="n">
-        <v>209.89</v>
+        <v>1232.72</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46174.22916666666</v>
+        <v>46177.72916666666</v>
       </c>
       <c r="B42" s="1" t="n">
-        <v>46174.25</v>
+        <v>46177.73958333334</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2135,16 +2135,16 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>4519.644</v>
+        <v>4476.887</v>
       </c>
       <c r="F42" t="n">
-        <v>4516.854</v>
+        <v>4478.535</v>
       </c>
       <c r="G42" t="n">
-        <v>4525.224</v>
+        <v>4471.942999999999</v>
       </c>
       <c r="H42" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2152,18 +2152,18 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>-27.9</v>
+        <v>-32.96</v>
       </c>
       <c r="K42" t="n">
-        <v>181.99</v>
+        <v>1199.76</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46174.41666666666</v>
+        <v>46178.01041666666</v>
       </c>
       <c r="B43" s="1" t="n">
-        <v>46174.42708333334</v>
+        <v>46178.02083333334</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -2176,35 +2176,35 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>4501.323</v>
+        <v>4457.399</v>
       </c>
       <c r="F43" t="n">
-        <v>4498.514</v>
+        <v>4455.657</v>
       </c>
       <c r="G43" t="n">
-        <v>4506.941000000001</v>
+        <v>4462.625000000001</v>
       </c>
       <c r="H43" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>-28.09</v>
+        <v>104.52</v>
       </c>
       <c r="K43" t="n">
-        <v>153.9</v>
+        <v>1304.28</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46175.125</v>
+        <v>46178.21875</v>
       </c>
       <c r="B44" s="1" t="n">
-        <v>46175.13541666666</v>
+        <v>46178.22916666666</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -2217,16 +2217,16 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>4488.012</v>
+        <v>4444.726</v>
       </c>
       <c r="F44" t="n">
-        <v>4489.012</v>
+        <v>4446.205</v>
       </c>
       <c r="G44" t="n">
-        <v>4486.012</v>
+        <v>4440.288999999999</v>
       </c>
       <c r="H44" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2234,22 +2234,22 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>20</v>
+        <v>88.73999999999999</v>
       </c>
       <c r="K44" t="n">
-        <v>173.9</v>
+        <v>1393.02</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>46175.38541666666</v>
+        <v>46178.69791666666</v>
       </c>
       <c r="B45" s="1" t="n">
-        <v>46175.40625</v>
+        <v>46178.70833333334</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2258,16 +2258,16 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>4526.834</v>
+        <v>4344.347</v>
       </c>
       <c r="F45" t="n">
-        <v>4529.791</v>
+        <v>4342.699</v>
       </c>
       <c r="G45" t="n">
-        <v>4520.919999999999</v>
+        <v>4349.291</v>
       </c>
       <c r="H45" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2275,18 +2275,18 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>-29.57</v>
+        <v>-32.96</v>
       </c>
       <c r="K45" t="n">
-        <v>144.33</v>
+        <v>1360.06</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>46175.6875</v>
+        <v>46178.80208333334</v>
       </c>
       <c r="B46" s="1" t="n">
-        <v>46175.70833333334</v>
+        <v>46178.8125</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -2299,601 +2299,27 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>4489.918</v>
+        <v>4323.674</v>
       </c>
       <c r="F46" t="n">
-        <v>4488.498</v>
+        <v>4321.588</v>
       </c>
       <c r="G46" t="n">
-        <v>4492.758</v>
+        <v>4329.932000000001</v>
       </c>
       <c r="H46" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>28.4</v>
+        <v>-41.72</v>
       </c>
       <c r="K46" t="n">
-        <v>172.73</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>46175.79166666666</v>
-      </c>
-      <c r="B47" s="1" t="n">
-        <v>46175.91666666666</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>4487.381</v>
-      </c>
-      <c r="F47" t="n">
-        <v>4491.498</v>
-      </c>
-      <c r="G47" t="n">
-        <v>4479.147000000002</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="J47" t="n">
-        <v>-41.17</v>
-      </c>
-      <c r="K47" t="n">
-        <v>131.56</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46176</v>
-      </c>
-      <c r="B48" s="1" t="n">
-        <v>46176.01041666666</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>4475.687</v>
-      </c>
-      <c r="F48" t="n">
-        <v>4480.146</v>
-      </c>
-      <c r="G48" t="n">
-        <v>4466.769</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="J48" t="n">
-        <v>-44.59</v>
-      </c>
-      <c r="K48" t="n">
-        <v>86.97</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>46176.09375</v>
-      </c>
-      <c r="B49" s="1" t="n">
-        <v>46176.10416666666</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>4478.584</v>
-      </c>
-      <c r="F49" t="n">
-        <v>4477.146</v>
-      </c>
-      <c r="G49" t="n">
-        <v>4481.46</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="J49" t="n">
-        <v>28.76</v>
-      </c>
-      <c r="K49" t="n">
-        <v>115.73</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>46176.11458333334</v>
-      </c>
-      <c r="B50" s="1" t="n">
-        <v>46176.125</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>4482.089</v>
-      </c>
-      <c r="F50" t="n">
-        <v>4480.574</v>
-      </c>
-      <c r="G50" t="n">
-        <v>4485.119000000001</v>
-      </c>
-      <c r="H50" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="J50" t="n">
-        <v>30.3</v>
-      </c>
-      <c r="K50" t="n">
-        <v>146.03</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>46176.28125</v>
-      </c>
-      <c r="B51" s="1" t="n">
-        <v>46176.29166666666</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>4462.83</v>
-      </c>
-      <c r="F51" t="n">
-        <v>4460.778</v>
-      </c>
-      <c r="G51" t="n">
-        <v>4466.933999999999</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="J51" t="n">
-        <v>41.04</v>
-      </c>
-      <c r="K51" t="n">
-        <v>187.07</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>46176.34375</v>
-      </c>
-      <c r="B52" s="1" t="n">
-        <v>46176.35416666666</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E52" t="n">
-        <v>4457.252</v>
-      </c>
-      <c r="F52" t="n">
-        <v>4454.977</v>
-      </c>
-      <c r="G52" t="n">
-        <v>4461.802000000001</v>
-      </c>
-      <c r="H52" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="J52" t="n">
-        <v>-22.75</v>
-      </c>
-      <c r="K52" t="n">
-        <v>164.32</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>46176.41666666666</v>
-      </c>
-      <c r="B53" s="1" t="n">
-        <v>46176.42708333334</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E53" t="n">
-        <v>4462.809</v>
-      </c>
-      <c r="F53" t="n">
-        <v>4460.778</v>
-      </c>
-      <c r="G53" t="n">
-        <v>4466.871</v>
-      </c>
-      <c r="H53" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="J53" t="n">
-        <v>-20.31</v>
-      </c>
-      <c r="K53" t="n">
-        <v>144.01</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>46176.61458333334</v>
-      </c>
-      <c r="B54" s="1" t="n">
-        <v>46176.625</v>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E54" t="n">
-        <v>4457.258</v>
-      </c>
-      <c r="F54" t="n">
-        <v>4454.977</v>
-      </c>
-      <c r="G54" t="n">
-        <v>4461.82</v>
-      </c>
-      <c r="H54" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="J54" t="n">
-        <v>-22.81</v>
-      </c>
-      <c r="K54" t="n">
-        <v>121.2</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>46176.92708333334</v>
-      </c>
-      <c r="B55" s="1" t="n">
-        <v>46176.9375</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E55" t="n">
-        <v>4433.806</v>
-      </c>
-      <c r="F55" t="n">
-        <v>4432.129</v>
-      </c>
-      <c r="G55" t="n">
-        <v>4437.159999999999</v>
-      </c>
-      <c r="H55" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="J55" t="n">
-        <v>33.54</v>
-      </c>
-      <c r="K55" t="n">
-        <v>154.74</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>46177.72916666666</v>
-      </c>
-      <c r="B56" s="1" t="n">
-        <v>46177.73958333334</v>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E56" t="n">
-        <v>4476.887</v>
-      </c>
-      <c r="F56" t="n">
-        <v>4478.535</v>
-      </c>
-      <c r="G56" t="n">
-        <v>4473.590999999999</v>
-      </c>
-      <c r="H56" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="J56" t="n">
-        <v>-16.48</v>
-      </c>
-      <c r="K56" t="n">
-        <v>138.26</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>46178.01041666666</v>
-      </c>
-      <c r="B57" s="1" t="n">
-        <v>46178.02083333334</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E57" t="n">
-        <v>4457.399</v>
-      </c>
-      <c r="F57" t="n">
-        <v>4455.657</v>
-      </c>
-      <c r="G57" t="n">
-        <v>4460.883000000001</v>
-      </c>
-      <c r="H57" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="J57" t="n">
-        <v>34.84</v>
-      </c>
-      <c r="K57" t="n">
-        <v>173.1</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>46178.21875</v>
-      </c>
-      <c r="B58" s="1" t="n">
-        <v>46178.22916666666</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E58" t="n">
-        <v>4444.726</v>
-      </c>
-      <c r="F58" t="n">
-        <v>4446.205</v>
-      </c>
-      <c r="G58" t="n">
-        <v>4441.767999999999</v>
-      </c>
-      <c r="H58" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="J58" t="n">
-        <v>29.58</v>
-      </c>
-      <c r="K58" t="n">
-        <v>202.68</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>46178.69791666666</v>
-      </c>
-      <c r="B59" s="1" t="n">
-        <v>46178.70833333334</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E59" t="n">
-        <v>4344.347</v>
-      </c>
-      <c r="F59" t="n">
-        <v>4342.699</v>
-      </c>
-      <c r="G59" t="n">
-        <v>4347.643</v>
-      </c>
-      <c r="H59" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="J59" t="n">
-        <v>-16.48</v>
-      </c>
-      <c r="K59" t="n">
-        <v>186.2</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>46178.80208333334</v>
-      </c>
-      <c r="B60" s="1" t="n">
-        <v>46178.8125</v>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>BOUNCE</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>4323.674</v>
-      </c>
-      <c r="F60" t="n">
-        <v>4321.588</v>
-      </c>
-      <c r="G60" t="n">
-        <v>4327.846</v>
-      </c>
-      <c r="H60" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="J60" t="n">
-        <v>-20.86</v>
-      </c>
-      <c r="K60" t="n">
-        <v>165.34</v>
+        <v>1318.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>